<commit_message>
M4 records, second pass: RC results, DEF-032, C. Burger's AI rows, TD-008 required
In place on the versions already in this PR (no new versions):
- RTM v0.11: the eight staging rows from the RC record (NFR-1.3, NFR-2.7, NFR-3.2 Met;
  NFR-1.11, NFR-3.1 Partially Met; NFR-2.1, NFR-2.4 Not Met, DEF-032; NFR-4.1 Not Met),
  the NFR-3.2 re-check on the domain, the A2 note and Status summary D9/D10.
  63 of 80 after the RC. 35 cells.
- Risk Register V0.9: RSK-010 and RSK-019 partly materialised at the RC, RSK-012, RSK-013
  and RSK-017 notes completed. 7 cells.
- AI Usage Register v0.15: C. Burger's two M4 rows (B97:I98), his wording unchanged. 16 cells.
- Technical Debt Register v0.4: TD-008's integration job is a required check in the dev
  ruleset since 18/10/2026; TD-007's owner is C. Burger, who repaid it in PR #123. 5 cells.

Each workbook was compared cell by cell against its committed version: every expected cell
matches and nothing else changed.
</commit_message>
<xml_diff>
--- a/docs/AI-Usage/AI Usage Register/AI Usage Register v0.15.xlsx
+++ b/docs/AI-Usage/AI Usage Register/AI Usage Register v0.15.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elind\m4-wt\records\docs\AI-Usage\AI Usage Register\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449D37F1-7018-456A-B4A6-1AD814667C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7746990F-0A8D-440F-9984-5274705A429E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="30912" windowHeight="17472" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AI Usage Register" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="461">
   <si>
     <t>AI Usage Register</t>
   </si>
@@ -1488,6 +1488,36 @@
   </si>
   <si>
     <t>The AI’s drafts needed 14 corrections before use, mostly figures and statuses that had changed since they were written; nothing was carried into PED v4.0 without being checked against the registers.</t>
+  </si>
+  <si>
+    <t>TD-008: run the 8 integration cases in CI</t>
+  </si>
+  <si>
+    <t>Drafted a sixth CI job that starts a single-node MongoDB 8.0 replica set on the runner, with no cluster credential, and runs the cases against it; the harness change that accepts that loopback host only when CI=true; and a step that fails the job if the cases were skipped. Wrote the expected result before the run: 40 tests, 25 pass, 15 fail (DEF-007 to DEF-011)</t>
+  </si>
+  <si>
+    <t>The run on PR #122 matched the prediction exactly: 40 tests, 25 pass, 15 fail, 0 skipped. Before that, the full suite with the harness change was unchanged from dev (199 tests, 191 pass), the host rule was tested against four URIs, and the skip guard failed the step when no database was given. After PR #136 the same job passed 40/40 on dev (run 39079571516)</t>
+  </si>
+  <si>
+    <t>Accepted with changes. Added as a non-required check while DEF-007 to DEF-011 still failed, so the known failures did not block other merges. After it passed 40/40 on dev, I made it a required check in the dev rule ruleset on 18/10/2026, which repays TD-008</t>
+  </si>
+  <si>
+    <t>TD Register v0.3 planned the known failures as expected failures. node:test has no expected-failure mode that fails when the test starts passing, so I made the job non-required instead of changing any assertion. MongoDB could not be downloaded in the drafting environment, so the replica set was first tried in CI itself</t>
+  </si>
+  <si>
+    <t>Pre-RC fixes : TD-007 OpenAPI tests parse the YAML, DEF-019 test titles, scripts README, .gitignore</t>
+  </si>
+  <si>
+    <t>Rewrote the two OpenAPI contract tests to parse the file with the yaml package as a dev dependency, and added a test for valid YAML, OpenAPI 3.x and resolving references. Corrected the two DEF-019 titles, the stale staging-marker line in the scripts README, and added ignores for the perf fixture file and staging.crt</t>
+  </si>
+  <si>
+    <t>Broke openapi.yaml four ways with the expected results written first: the old tests passed on three of the four, the new ones failed on all four, and the file was restored and hash-checked each time. Full suite 200 tests, 192 pass; ESLint clean; production audit 0 vulnerabilities; the lockfile change is only the yaml package; the ignore rules were tested in an empty repo</t>
+  </si>
+  <si>
+    <t>Accepted. A YAML parser rather than a full OpenAPI validator, with the limit stated in the test headers. Split into three commits, one per fix</t>
+  </si>
+  <si>
+    <t>The negative verification ran in a scratch copy, not in my checkout, and the evidence file says so. One commit message was joined to old text by mistake and was amended before review</t>
   </si>
 </sst>
 </file>
@@ -1657,7 +1687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1718,9 +1748,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4203,401 +4230,435 @@
     </row>
     <row r="83" spans="2:9" ht="115.2">
       <c r="B83" s="15">
+        <f t="shared" ref="B83:B96" si="3">DATE(2026,10,17)</f>
+        <v>46312</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="F83" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="H83" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="I83" s="5" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="84" spans="2:9" ht="72">
+      <c r="B84" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="F84" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="I84" s="5" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="85" spans="2:9" ht="100.8">
+      <c r="B85" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="F85" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="H85" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="86" spans="2:9" ht="86.4">
+      <c r="B86" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="F86" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="I86" s="5" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="87" spans="2:9" ht="86.4">
+      <c r="B87" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E87" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="F87" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="G87" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="I87" s="5" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="88" spans="2:9" ht="72">
+      <c r="B88" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="F88" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="H88" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="I88" s="5" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="89" spans="2:9" ht="86.4">
+      <c r="B89" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="F89" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="H89" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="I89" s="5" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="90" spans="2:9" ht="115.2">
+      <c r="B90" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D90" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="I90" s="5" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="91" spans="2:9" ht="115.2">
+      <c r="B91" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="F91" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="H91" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="I91" s="5" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="92" spans="2:9" ht="100.8">
+      <c r="B92" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D92" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="H92" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="I92" s="5" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="93" spans="2:9" ht="86.4">
+      <c r="B93" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C93" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="H93" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="I93" s="5" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="94" spans="2:9" ht="43.2">
+      <c r="B94" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="G94" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="H94" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="I94" s="5" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="95" spans="2:9" ht="72">
+      <c r="B95" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="F95" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H95" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="96" spans="2:9" ht="144">
+      <c r="B96" s="15">
+        <f t="shared" si="3"/>
+        <v>46312</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="H96" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="I96" s="5" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="97" spans="2:9" ht="115.2">
+      <c r="B97" s="15">
         <f>DATE(2026,10,17)</f>
         <v>46312</v>
       </c>
-      <c r="C83" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D83" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="F83" s="21" t="s">
-        <v>402</v>
-      </c>
-      <c r="G83" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="H83" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="I83" s="5" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="84" spans="2:9" ht="72">
-      <c r="B84" s="15">
+      <c r="C97" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="G97" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="H97" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="I97" s="5" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="98" spans="2:9" ht="115.2">
+      <c r="B98" s="15">
         <f>DATE(2026,10,17)</f>
         <v>46312</v>
       </c>
-      <c r="C84" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D84" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="F84" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="G84" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="H84" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="I84" s="5" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="85" spans="2:9" ht="100.8">
-      <c r="B85" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D85" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="F85" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="H85" s="21" t="s">
-        <v>448</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="86" spans="2:9" ht="86.4">
-      <c r="B86" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D86" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="F86" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="G86" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="H86" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="I86" s="5" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="87" spans="2:9" ht="86.4">
-      <c r="B87" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D87" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="F87" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="G87" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="H87" s="21" t="s">
-        <v>449</v>
-      </c>
-      <c r="I87" s="21" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="88" spans="2:9" ht="72">
-      <c r="B88" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D88" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="F88" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="G88" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="H88" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="I88" s="5" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="89" spans="2:9" ht="86.4">
-      <c r="B89" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D89" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="F89" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="G89" s="5" t="s">
-        <v>410</v>
-      </c>
-      <c r="H89" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="I89" s="5" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="90" spans="2:9" ht="115.2">
-      <c r="B90" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D90" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="F90" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="G90" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="H90" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="I90" s="5" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="91" spans="2:9" ht="115.2">
-      <c r="B91" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D91" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="G91" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="H91" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="I91" s="5" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="92" spans="2:9" ht="100.8">
-      <c r="B92" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D92" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="F92" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="G92" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="H92" s="5" t="s">
-        <v>426</v>
-      </c>
-      <c r="I92" s="5" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="93" spans="2:9" ht="86.4">
-      <c r="B93" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D93" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="F93" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="G93" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="H93" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="I93" s="5" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="94" spans="2:9" ht="43.2">
-      <c r="B94" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="F94" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="G94" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="H94" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="I94" s="5" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="95" spans="2:9" ht="72">
-      <c r="B95" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D95" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="F95" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="G95" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="H95" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="I95" s="5" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="96" spans="2:9" ht="144">
-      <c r="B96" s="15">
-        <f>DATE(2026,10,17)</f>
-        <v>46312</v>
-      </c>
-      <c r="C96" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D96" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="F96" s="5" t="s">
-        <v>444</v>
-      </c>
-      <c r="G96" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="H96" s="5" t="s">
-        <v>446</v>
-      </c>
-      <c r="I96" s="5" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="97" spans="2:9">
-      <c r="B97" s="8"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="7"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
-      <c r="I97" s="5"/>
-    </row>
-    <row r="98" spans="2:9">
-      <c r="B98" s="8"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="7"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
-      <c r="I98" s="5"/>
+      <c r="C98" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="H98" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>460</v>
+      </c>
     </row>
     <row r="99" spans="2:9">
       <c r="B99" s="8"/>

</xml_diff>